<commit_message>
Improved accuracy, added QR & manual attendance features, UI enhancements and report fixes
</commit_message>
<xml_diff>
--- a/backend/attendance_report.xlsx
+++ b/backend/attendance_report.xlsx
@@ -29,12 +29,24 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -55,11 +67,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,12 +439,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C71"/>
+  <dimension ref="A1:D71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -446,1195 +461,1550 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Timestamp</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>23wh1a6601</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24 00:06:02</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>23wh1a6602</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>23wh1a6603</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>23wh1a6604</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>23wh1a6605</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>face</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24 00:05:28</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>23wh1a6606</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>23wh1a6607</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>23wh1a6608</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>23wh1a6609</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>23wh1a6610</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>23wh1a6611</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>23wh1a6612</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>23wh1a6613</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>23wh1a6614</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>23wh1a6615</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>Present</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>2026-03-22 19:33:44</t>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>face</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24 00:05:28</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>23wh1a6616</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>23wh1a6617</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>23wh1a6618</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>23wh1a6619</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>23wh1a6620</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>23wh1a6621</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>23wh1a6622</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>23wh1a6623</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>23wh1a6624</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t>Present</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>2026-03-22 19:33:44</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>23wh1a6623</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>23wh1a6624</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>qr</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24 00:06:37</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>23wh1a6625</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>23wh1a6626</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>23wh1a6627</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>23wh1a6628</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>23wh1a6629</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>23wh1a6630</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>23wh1a6631</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>23wh1a6632</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="3" t="inlineStr">
         <is>
           <t>23wh1a6633</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>23wh1a6634</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="3" t="inlineStr">
         <is>
           <t>23wh1a6635</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>23wh1a6636</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="3" t="inlineStr">
         <is>
           <t>23wh1a6637</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>23wh1a6638</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>23wh1a6639</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>23wh1a6640</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
         <is>
           <t>Present</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>2026-03-22 19:33:44</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>23wh1a6639</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>23wh1a6640</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24 00:06:02</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="A42" s="3" t="inlineStr">
         <is>
           <t>23wh1a6641</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
+      <c r="A43" s="3" t="inlineStr">
         <is>
           <t>23wh1a6642</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
+      <c r="A44" s="3" t="inlineStr">
         <is>
           <t>23wh1a6643</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
+      <c r="A45" s="3" t="inlineStr">
         <is>
           <t>23wh1a6644</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
+      <c r="A46" s="3" t="inlineStr">
         <is>
           <t>23wh1a6645</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
+      <c r="A47" s="3" t="inlineStr">
         <is>
           <t>23wh1a6646</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
+      <c r="A48" s="3" t="inlineStr">
         <is>
           <t>23wh1a6647</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
+      <c r="A49" s="3" t="inlineStr">
         <is>
           <t>23wh1a6648</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>23wh1a6649</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>face</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24 00:05:28</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
+      <c r="A51" s="3" t="inlineStr">
         <is>
           <t>23wh1a6650</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
+      <c r="A52" s="3" t="inlineStr">
         <is>
           <t>23wh1a6651</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
+      <c r="A53" s="2" t="inlineStr">
         <is>
           <t>23wh1a6652</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>face</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24 00:05:28</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
+      <c r="A54" s="3" t="inlineStr">
         <is>
           <t>23wh1a6653</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
+      <c r="A55" s="3" t="inlineStr">
         <is>
           <t>23wh1a6654</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
+      <c r="A56" s="3" t="inlineStr">
         <is>
           <t>23wh1a6655</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
+      <c r="A57" s="3" t="inlineStr">
         <is>
           <t>23wh1a6656</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
+      <c r="A58" s="3" t="inlineStr">
         <is>
           <t>23wh1a6657</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr">
+      <c r="A59" s="3" t="inlineStr">
         <is>
           <t>23wh1a6658</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr">
+      <c r="A60" s="3" t="inlineStr">
         <is>
           <t>23wh1a6659</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr">
+      <c r="A61" s="3" t="inlineStr">
         <is>
           <t>23wh1a6660</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr">
+      <c r="A62" s="3" t="inlineStr">
         <is>
           <t>23wh1a6661</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
+      <c r="A63" s="3" t="inlineStr">
         <is>
           <t>23wh1a6662</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr">
+      <c r="A64" s="3" t="inlineStr">
         <is>
           <t>23wh1a6663</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr">
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>24wh5a6601</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>24wh5a6602</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>24wh5a6603</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>24wh5a6604</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
         <is>
           <t>Present</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>2026-03-22 19:33:44</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>24wh5a6601</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>24wh5a6602</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>24wh5a6603</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>24wh5a6604</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>face</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24 00:05:28</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
+      <c r="A69" s="3" t="inlineStr">
         <is>
           <t>24wh5a6605</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" t="inlineStr">
+      <c r="A70" s="3" t="inlineStr">
         <is>
           <t>24wh5a6606</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" t="inlineStr">
+      <c r="A71" s="3" t="inlineStr">
         <is>
           <t>24wh5a6607</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
Update: AI Attendance System
</commit_message>
<xml_diff>
--- a/backend/attendance_report.xlsx
+++ b/backend/attendance_report.xlsx
@@ -483,12 +483,12 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>manual</t>
+          <t>face,manual</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-03-24 00:06:02</t>
+          <t>2026-03-24 21:29:28</t>
         </is>
       </c>
     </row>
@@ -571,12 +571,12 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>face</t>
+          <t>manual</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-03-24 00:05:28</t>
+          <t>2026-03-24 21:30:53</t>
         </is>
       </c>
     </row>
@@ -691,24 +691,24 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>23wh1a6611</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>face</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24 21:29:28</t>
         </is>
       </c>
     </row>
@@ -791,12 +791,12 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>face</t>
+          <t>manual</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>2026-03-24 00:05:28</t>
+          <t>2026-03-24 21:30:53</t>
         </is>
       </c>
     </row>
@@ -933,46 +933,46 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>23wh1a6622</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24 21:30:53</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>23wh1a6623</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>face</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24 21:29:28</t>
         </is>
       </c>
     </row>
@@ -989,12 +989,12 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>qr</t>
+          <t>manual</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>2026-03-24 00:06:37</t>
+          <t>2026-03-24 21:30:53</t>
         </is>
       </c>
     </row>
@@ -1021,24 +1021,24 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>23wh1a6626</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>face</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24 21:29:28</t>
         </is>
       </c>
     </row>
@@ -1153,46 +1153,46 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="3" t="inlineStr">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>23wh1a6632</t>
         </is>
       </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D33" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24 21:30:53</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="3" t="inlineStr">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>23wh1a6633</t>
         </is>
       </c>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C34" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>qr</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24 21:37:16</t>
         </is>
       </c>
     </row>
@@ -1346,7 +1346,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>2026-03-24 00:06:02</t>
+          <t>2026-03-24 21:30:53</t>
         </is>
       </c>
     </row>
@@ -1395,24 +1395,24 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="3" t="inlineStr">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>23wh1a6643</t>
         </is>
       </c>
-      <c r="B44" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C44" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D44" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>manual,qr</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24 21:30:53</t>
         </is>
       </c>
     </row>
@@ -1461,24 +1461,24 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="3" t="inlineStr">
+      <c r="A47" s="2" t="inlineStr">
         <is>
           <t>23wh1a6646</t>
         </is>
       </c>
-      <c r="B47" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C47" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D47" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>face</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24 21:29:28</t>
         </is>
       </c>
     </row>
@@ -1527,24 +1527,24 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="inlineStr">
+      <c r="A50" s="3" t="inlineStr">
         <is>
           <t>23wh1a6649</t>
         </is>
       </c>
-      <c r="B50" s="2" t="inlineStr">
-        <is>
-          <t>Present</t>
-        </is>
-      </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>face</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>2026-03-24 00:05:28</t>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1610,7 +1610,7 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>2026-03-24 00:05:28</t>
+          <t>2026-03-24 21:29:28</t>
         </is>
       </c>
     </row>
@@ -1703,24 +1703,24 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="3" t="inlineStr">
+      <c r="A58" s="2" t="inlineStr">
         <is>
           <t>23wh1a6657</t>
         </is>
       </c>
-      <c r="B58" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C58" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D58" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>face</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24 21:29:28</t>
         </is>
       </c>
     </row>
@@ -1769,24 +1769,24 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="3" t="inlineStr">
+      <c r="A61" s="2" t="inlineStr">
         <is>
           <t>23wh1a6660</t>
         </is>
       </c>
-      <c r="B61" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C61" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D61" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>qr</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24 21:36:23</t>
         </is>
       </c>
     </row>
@@ -1813,46 +1813,46 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="3" t="inlineStr">
+      <c r="A63" s="2" t="inlineStr">
         <is>
           <t>23wh1a6662</t>
         </is>
       </c>
-      <c r="B63" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C63" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D63" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>face</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24 21:29:28</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="3" t="inlineStr">
+      <c r="A64" s="2" t="inlineStr">
         <is>
           <t>23wh1a6663</t>
         </is>
       </c>
-      <c r="B64" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C64" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D64" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24 21:30:53</t>
         </is>
       </c>
     </row>
@@ -1901,46 +1901,46 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="3" t="inlineStr">
+      <c r="A67" s="2" t="inlineStr">
         <is>
           <t>24wh5a6603</t>
         </is>
       </c>
-      <c r="B67" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C67" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D67" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Present</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>face</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-24 21:29:28</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="inlineStr">
+      <c r="A68" s="3" t="inlineStr">
         <is>
           <t>24wh5a6604</t>
         </is>
       </c>
-      <c r="B68" s="2" t="inlineStr">
-        <is>
-          <t>Present</t>
-        </is>
-      </c>
-      <c r="C68" s="2" t="inlineStr">
-        <is>
-          <t>face</t>
-        </is>
-      </c>
-      <c r="D68" s="2" t="inlineStr">
-        <is>
-          <t>2026-03-24 00:05:28</t>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
UI Changes: dashboard count, download options
</commit_message>
<xml_diff>
--- a/backend/attendance_report.xlsx
+++ b/backend/attendance_report.xlsx
@@ -38,14 +38,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-        <bgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
-        <bgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -478,81 +478,81 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Present</t>
+          <t>Absent</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>face,manual</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2026-03-24 21:29:28</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>23wh1a6602</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>23wh1a6603</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>23wh1a6604</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -566,125 +566,125 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Present</t>
+          <t>Absent</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>manual</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>2026-03-24 21:30:53</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>23wh1a6606</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>23wh1a6607</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>23wh1a6608</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>23wh1a6609</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>23wh1a6610</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -698,81 +698,81 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Present</t>
+          <t>Absent</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>face</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>2026-03-24 21:29:28</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>23wh1a6612</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>23wh1a6613</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>23wh1a6614</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -786,147 +786,147 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Present</t>
+          <t>Absent</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>manual</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>2026-03-24 21:30:53</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>23wh1a6616</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>23wh1a6617</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>23wh1a6618</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>23wh1a6619</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>23wh1a6620</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>23wh1a6621</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -940,17 +940,17 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Present</t>
+          <t>Absent</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>manual</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>2026-03-24 21:30:53</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -962,17 +962,17 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Present</t>
+          <t>Absent</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>face</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>2026-03-24 21:29:28</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -984,37 +984,37 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Present</t>
+          <t>Absent</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>manual</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>2026-03-24 21:30:53</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>23wh1a6625</t>
         </is>
       </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1028,125 +1028,125 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Present</t>
+          <t>Absent</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>face</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>2026-03-24 21:29:28</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="inlineStr">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>23wh1a6627</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>23wh1a6628</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="inlineStr">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>23wh1a6629</t>
         </is>
       </c>
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>23wh1a6630</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D31" s="3" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="inlineStr">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>23wh1a6631</t>
         </is>
       </c>
-      <c r="B32" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D32" s="3" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1160,17 +1160,17 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Present</t>
+          <t>Absent</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>manual</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>2026-03-24 21:30:53</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1182,213 +1182,213 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>23wh1a6634</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>23wh1a6635</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>23wh1a6636</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>23wh1a6637</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>23wh1a6638</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>23wh1a6639</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>23wh1a6640</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
           <t>Present</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>qr</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>2026-03-24 21:37:16</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t>23wh1a6634</t>
-        </is>
-      </c>
-      <c r="B35" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D35" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="3" t="inlineStr">
-        <is>
-          <t>23wh1a6635</t>
-        </is>
-      </c>
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D36" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="3" t="inlineStr">
-        <is>
-          <t>23wh1a6636</t>
-        </is>
-      </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D37" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="3" t="inlineStr">
-        <is>
-          <t>23wh1a6637</t>
-        </is>
-      </c>
-      <c r="B38" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C38" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D38" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>23wh1a6638</t>
-        </is>
-      </c>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D39" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="3" t="inlineStr">
-        <is>
-          <t>23wh1a6639</t>
-        </is>
-      </c>
-      <c r="B40" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C40" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D40" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>23wh1a6640</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>Present</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="inlineStr">
+      <c r="C41" s="3" t="inlineStr">
         <is>
           <t>manual</t>
         </is>
       </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>2026-03-24 21:30:53</t>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>2026-04-23 12:42:13</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="3" t="inlineStr">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>23wh1a6641</t>
         </is>
       </c>
-      <c r="B42" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C42" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D42" s="3" t="inlineStr">
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="3" t="inlineStr">
+      <c r="A43" s="2" t="inlineStr">
         <is>
           <t>23wh1a6642</t>
         </is>
       </c>
-      <c r="B43" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D43" s="3" t="inlineStr">
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1402,59 +1402,59 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Present</t>
+          <t>Absent</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>manual,qr</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>2026-03-24 21:30:53</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="3" t="inlineStr">
+      <c r="A45" s="2" t="inlineStr">
         <is>
           <t>23wh1a6644</t>
         </is>
       </c>
-      <c r="B45" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C45" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D45" s="3" t="inlineStr">
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="3" t="inlineStr">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t>23wh1a6645</t>
         </is>
       </c>
-      <c r="B46" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C46" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D46" s="3" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1468,125 +1468,125 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Present</t>
+          <t>Absent</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>face</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>2026-03-24 21:29:28</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="3" t="inlineStr">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>23wh1a6647</t>
         </is>
       </c>
-      <c r="B48" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C48" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D48" s="3" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="3" t="inlineStr">
+      <c r="A49" s="2" t="inlineStr">
         <is>
           <t>23wh1a6648</t>
         </is>
       </c>
-      <c r="B49" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C49" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D49" s="3" t="inlineStr">
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="3" t="inlineStr">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>23wh1a6649</t>
         </is>
       </c>
-      <c r="B50" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C50" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D50" s="3" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="3" t="inlineStr">
+      <c r="A51" s="2" t="inlineStr">
         <is>
           <t>23wh1a6650</t>
         </is>
       </c>
-      <c r="B51" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C51" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D51" s="3" t="inlineStr">
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="3" t="inlineStr">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>23wh1a6651</t>
         </is>
       </c>
-      <c r="B52" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C52" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D52" s="3" t="inlineStr">
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1600,103 +1600,103 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Present</t>
+          <t>Absent</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>face</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>2026-03-24 21:29:28</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="3" t="inlineStr">
+      <c r="A54" s="2" t="inlineStr">
         <is>
           <t>23wh1a6653</t>
         </is>
       </c>
-      <c r="B54" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C54" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D54" s="3" t="inlineStr">
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="3" t="inlineStr">
+      <c r="A55" s="2" t="inlineStr">
         <is>
           <t>23wh1a6654</t>
         </is>
       </c>
-      <c r="B55" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C55" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D55" s="3" t="inlineStr">
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="3" t="inlineStr">
+      <c r="A56" s="2" t="inlineStr">
         <is>
           <t>23wh1a6655</t>
         </is>
       </c>
-      <c r="B56" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C56" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D56" s="3" t="inlineStr">
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="3" t="inlineStr">
+      <c r="A57" s="2" t="inlineStr">
         <is>
           <t>23wh1a6656</t>
         </is>
       </c>
-      <c r="B57" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C57" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D57" s="3" t="inlineStr">
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1710,59 +1710,59 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Present</t>
+          <t>Absent</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>face</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>2026-03-24 21:29:28</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="3" t="inlineStr">
+      <c r="A59" s="2" t="inlineStr">
         <is>
           <t>23wh1a6658</t>
         </is>
       </c>
-      <c r="B59" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C59" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D59" s="3" t="inlineStr">
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="3" t="inlineStr">
+      <c r="A60" s="2" t="inlineStr">
         <is>
           <t>23wh1a6659</t>
         </is>
       </c>
-      <c r="B60" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C60" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D60" s="3" t="inlineStr">
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1776,37 +1776,37 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Present</t>
+          <t>Absent</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>qr</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
         <is>
-          <t>2026-03-24 21:36:23</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="3" t="inlineStr">
+      <c r="A62" s="2" t="inlineStr">
         <is>
           <t>23wh1a6661</t>
         </is>
       </c>
-      <c r="B62" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C62" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D62" s="3" t="inlineStr">
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1820,17 +1820,17 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Present</t>
+          <t>Absent</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>face</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t>2026-03-24 21:29:28</t>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -1842,59 +1842,59 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Present</t>
+          <t>Absent</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>manual</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>2026-03-24 21:30:53</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="3" t="inlineStr">
+      <c r="A65" s="2" t="inlineStr">
         <is>
           <t>24wh5a6601</t>
         </is>
       </c>
-      <c r="B65" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C65" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D65" s="3" t="inlineStr">
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="3" t="inlineStr">
+      <c r="A66" s="2" t="inlineStr">
         <is>
           <t>24wh5a6602</t>
         </is>
       </c>
-      <c r="B66" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C66" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D66" s="3" t="inlineStr">
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1908,103 +1908,103 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>Present</t>
+          <t>Absent</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>face</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
         <is>
-          <t>2026-03-24 21:29:28</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="3" t="inlineStr">
+      <c r="A68" s="2" t="inlineStr">
         <is>
           <t>24wh5a6604</t>
         </is>
       </c>
-      <c r="B68" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C68" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D68" s="3" t="inlineStr">
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="3" t="inlineStr">
+      <c r="A69" s="2" t="inlineStr">
         <is>
           <t>24wh5a6605</t>
         </is>
       </c>
-      <c r="B69" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C69" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D69" s="3" t="inlineStr">
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="3" t="inlineStr">
+      <c r="A70" s="2" t="inlineStr">
         <is>
           <t>24wh5a6606</t>
         </is>
       </c>
-      <c r="B70" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C70" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D70" s="3" t="inlineStr">
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="3" t="inlineStr">
+      <c r="A71" s="2" t="inlineStr">
         <is>
           <t>24wh5a6607</t>
         </is>
       </c>
-      <c r="B71" s="3" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C71" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D71" s="3" t="inlineStr">
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
feat: Google OAuth, live stats, PiP animation, fixes
</commit_message>
<xml_diff>
--- a/backend/attendance_report.xlsx
+++ b/backend/attendance_report.xlsx
@@ -38,14 +38,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
-        <bgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-        <bgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -478,81 +478,81 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Absent</t>
+          <t>Present</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>face</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-06-24 15:19:35</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>23wh1a6602</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>23wh1a6603</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>23wh1a6604</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -566,81 +566,81 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Absent</t>
+          <t>Present</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>face</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-06-24 15:19:35</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>23wh1a6606</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>23wh1a6607</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>23wh1a6608</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -654,213 +654,213 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Absent</t>
+          <t>Present</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>face</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-06-24 15:19:35</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>23wh1a6610</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>23wh1a6611</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>23wh1a6612</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>23wh1a6613</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>23wh1a6614</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>23wh1a6615</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>23wh1a6616</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>23wh1a6617</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>23wh1a6618</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -874,455 +874,455 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Absent</t>
+          <t>Present</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>face</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-06-24 15:19:35</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>23wh1a6620</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>23wh1a6621</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>23wh1a6622</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>23wh1a6623</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>23wh1a6624</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>23wh1a6625</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>23wh1a6626</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>23wh1a6627</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>23wh1a6628</t>
         </is>
       </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>23wh1a6629</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>23wh1a6630</t>
         </is>
       </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>23wh1a6631</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C32" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>23wh1a6632</t>
         </is>
       </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D33" s="2" t="inlineStr">
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="A34" s="3" t="inlineStr">
         <is>
           <t>23wh1a6633</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>23wh1a6634</t>
         </is>
       </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="A36" s="3" t="inlineStr">
         <is>
           <t>23wh1a6635</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>23wh1a6636</t>
         </is>
       </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="A38" s="3" t="inlineStr">
         <is>
           <t>23wh1a6637</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>23wh1a6638</t>
         </is>
       </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="A40" s="3" t="inlineStr">
         <is>
           <t>23wh1a6639</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1336,103 +1336,103 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Present</t>
+          <t>Absent</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>manual</t>
+          <t>-</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>2026-04-23 12:42:13</t>
+          <t>-</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="A42" s="3" t="inlineStr">
         <is>
           <t>23wh1a6641</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="inlineStr">
+      <c r="A43" s="3" t="inlineStr">
         <is>
           <t>23wh1a6642</t>
         </is>
       </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="inlineStr">
+      <c r="A44" s="3" t="inlineStr">
         <is>
           <t>23wh1a6643</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
+      <c r="A45" s="3" t="inlineStr">
         <is>
           <t>23wh1a6644</t>
         </is>
       </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr">
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1446,169 +1446,169 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Absent</t>
+          <t>Present</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>face</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-06-24 15:19:35</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="inlineStr">
+      <c r="A47" s="3" t="inlineStr">
         <is>
           <t>23wh1a6646</t>
         </is>
       </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="inlineStr">
+      <c r="A48" s="3" t="inlineStr">
         <is>
           <t>23wh1a6647</t>
         </is>
       </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="inlineStr">
+      <c r="A49" s="3" t="inlineStr">
         <is>
           <t>23wh1a6648</t>
         </is>
       </c>
-      <c r="B49" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C49" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D49" s="2" t="inlineStr">
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="inlineStr">
+      <c r="A50" s="3" t="inlineStr">
         <is>
           <t>23wh1a6649</t>
         </is>
       </c>
-      <c r="B50" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr">
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="inlineStr">
+      <c r="A51" s="3" t="inlineStr">
         <is>
           <t>23wh1a6650</t>
         </is>
       </c>
-      <c r="B51" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C51" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D51" s="2" t="inlineStr">
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="inlineStr">
+      <c r="A52" s="3" t="inlineStr">
         <is>
           <t>23wh1a6651</t>
         </is>
       </c>
-      <c r="B52" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C52" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D52" s="2" t="inlineStr">
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="inlineStr">
+      <c r="A53" s="3" t="inlineStr">
         <is>
           <t>23wh1a6652</t>
         </is>
       </c>
-      <c r="B53" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C53" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D53" s="2" t="inlineStr">
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1622,257 +1622,257 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Absent</t>
+          <t>Present</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>face</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-06-24 15:19:35</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="inlineStr">
+      <c r="A55" s="3" t="inlineStr">
         <is>
           <t>23wh1a6654</t>
         </is>
       </c>
-      <c r="B55" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C55" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D55" s="2" t="inlineStr">
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="inlineStr">
+      <c r="A56" s="3" t="inlineStr">
         <is>
           <t>23wh1a6655</t>
         </is>
       </c>
-      <c r="B56" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C56" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D56" s="2" t="inlineStr">
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="inlineStr">
+      <c r="A57" s="3" t="inlineStr">
         <is>
           <t>23wh1a6656</t>
         </is>
       </c>
-      <c r="B57" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C57" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D57" s="2" t="inlineStr">
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="inlineStr">
+      <c r="A58" s="3" t="inlineStr">
         <is>
           <t>23wh1a6657</t>
         </is>
       </c>
-      <c r="B58" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C58" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D58" s="2" t="inlineStr">
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="inlineStr">
+      <c r="A59" s="3" t="inlineStr">
         <is>
           <t>23wh1a6658</t>
         </is>
       </c>
-      <c r="B59" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C59" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D59" s="2" t="inlineStr">
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="inlineStr">
+      <c r="A60" s="3" t="inlineStr">
         <is>
           <t>23wh1a6659</t>
         </is>
       </c>
-      <c r="B60" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C60" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D60" s="2" t="inlineStr">
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="inlineStr">
+      <c r="A61" s="3" t="inlineStr">
         <is>
           <t>23wh1a6660</t>
         </is>
       </c>
-      <c r="B61" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C61" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D61" s="2" t="inlineStr">
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="inlineStr">
+      <c r="A62" s="3" t="inlineStr">
         <is>
           <t>23wh1a6661</t>
         </is>
       </c>
-      <c r="B62" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C62" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D62" s="2" t="inlineStr">
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="inlineStr">
+      <c r="A63" s="3" t="inlineStr">
         <is>
           <t>23wh1a6662</t>
         </is>
       </c>
-      <c r="B63" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C63" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D63" s="2" t="inlineStr">
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="inlineStr">
+      <c r="A64" s="3" t="inlineStr">
         <is>
           <t>23wh1a6663</t>
         </is>
       </c>
-      <c r="B64" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C64" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D64" s="2" t="inlineStr">
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="inlineStr">
+      <c r="A65" s="3" t="inlineStr">
         <is>
           <t>24wh5a6601</t>
         </is>
       </c>
-      <c r="B65" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C65" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D65" s="2" t="inlineStr">
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1886,125 +1886,125 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Absent</t>
+          <t>Present</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>face</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-06-24 15:19:35</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="inlineStr">
+      <c r="A67" s="3" t="inlineStr">
         <is>
           <t>24wh5a6603</t>
         </is>
       </c>
-      <c r="B67" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C67" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D67" s="2" t="inlineStr">
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="inlineStr">
+      <c r="A68" s="3" t="inlineStr">
         <is>
           <t>24wh5a6604</t>
         </is>
       </c>
-      <c r="B68" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C68" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D68" s="2" t="inlineStr">
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="inlineStr">
+      <c r="A69" s="3" t="inlineStr">
         <is>
           <t>24wh5a6605</t>
         </is>
       </c>
-      <c r="B69" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C69" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D69" s="2" t="inlineStr">
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="inlineStr">
+      <c r="A70" s="3" t="inlineStr">
         <is>
           <t>24wh5a6606</t>
         </is>
       </c>
-      <c r="B70" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C70" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D70" s="2" t="inlineStr">
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="2" t="inlineStr">
+      <c r="A71" s="3" t="inlineStr">
         <is>
           <t>24wh5a6607</t>
         </is>
       </c>
-      <c r="B71" s="2" t="inlineStr">
-        <is>
-          <t>Absent</t>
-        </is>
-      </c>
-      <c r="C71" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D71" s="2" t="inlineStr">
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>Absent</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>